<commit_message>
First successful run. Much refining to do
</commit_message>
<xml_diff>
--- a/input_files/capacity_limits.xlsx
+++ b/input_files/capacity_limits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/CODERS scripts/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{AD9299FD-BE0E-4A8B-BE4E-54B5B8BEA38F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19E2286A-1D9B-4C55-8259-3715807E5FC6}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{AD9299FD-BE0E-4A8B-BE4E-54B5B8BEA38F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EA1E23B-CEE6-4503-B61E-F57C96A666B6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{34B1FE10-2B49-41F7-8CAC-48335CB056E6}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11385" xr2:uid="{34B1FE10-2B49-41F7-8CAC-48335CB056E6}"/>
   </bookViews>
   <sheets>
     <sheet name="ON" sheetId="1" r:id="rId1"/>
@@ -34,28 +34,121 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Sets the maximum capacity of technologies by period.</t>
   </si>
   <si>
-    <t>E_WIND_ON-NEW-1</t>
-  </si>
-  <si>
     <t>tech</t>
   </si>
   <si>
     <t>max MW per period</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-1</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-2</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-3</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-4</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-5</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-6</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-7</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-8</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-9</t>
+  </si>
+  <si>
+    <t>E_SOL_PV-NEW-10</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-1</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-2</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-3</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-4</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-5</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-6</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-7</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-8</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-9</t>
+  </si>
+  <si>
+    <t>E_HYD_ROR-NEW-10</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-1</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-2</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-3</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-4</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-5</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-6</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-7</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-8</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-9</t>
+  </si>
+  <si>
+    <t>E_WND_ON-NEW-10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -397,7 +490,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9D36A0F-FD90-42AA-87C7-33795DBA1E16}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.140625" customWidth="1"/>
@@ -410,12 +503,12 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3">
         <v>2025</v>
@@ -438,10 +531,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="C4">
         <v>1000</v>
@@ -459,7 +552,675 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5">
+        <v>1000</v>
+      </c>
+      <c r="C5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>1000</v>
+      </c>
+      <c r="E5">
+        <v>1000</v>
+      </c>
+      <c r="F5">
+        <v>1000</v>
+      </c>
+      <c r="G5">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6">
+        <v>1000</v>
+      </c>
+      <c r="C6">
+        <v>1000</v>
+      </c>
+      <c r="D6">
+        <v>1000</v>
+      </c>
+      <c r="E6">
+        <v>1000</v>
+      </c>
+      <c r="F6">
+        <v>1000</v>
+      </c>
+      <c r="G6">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7">
+        <v>1000</v>
+      </c>
+      <c r="C7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>1000</v>
+      </c>
+      <c r="E7">
+        <v>1000</v>
+      </c>
+      <c r="F7">
+        <v>1000</v>
+      </c>
+      <c r="G7">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8">
+        <v>1000</v>
+      </c>
+      <c r="C8">
+        <v>1000</v>
+      </c>
+      <c r="D8">
+        <v>1000</v>
+      </c>
+      <c r="E8">
+        <v>1000</v>
+      </c>
+      <c r="F8">
+        <v>1000</v>
+      </c>
+      <c r="G8">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9">
+        <v>1000</v>
+      </c>
+      <c r="C9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>1000</v>
+      </c>
+      <c r="E9">
+        <v>1000</v>
+      </c>
+      <c r="F9">
+        <v>1000</v>
+      </c>
+      <c r="G9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10">
+        <v>1000</v>
+      </c>
+      <c r="C10">
+        <v>1000</v>
+      </c>
+      <c r="D10">
+        <v>1000</v>
+      </c>
+      <c r="E10">
+        <v>1000</v>
+      </c>
+      <c r="F10">
+        <v>1000</v>
+      </c>
+      <c r="G10">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11">
+        <v>1000</v>
+      </c>
+      <c r="C11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>1000</v>
+      </c>
+      <c r="E11">
+        <v>1000</v>
+      </c>
+      <c r="F11">
+        <v>1000</v>
+      </c>
+      <c r="G11">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12">
+        <v>1000</v>
+      </c>
+      <c r="C12">
+        <v>1000</v>
+      </c>
+      <c r="D12">
+        <v>1000</v>
+      </c>
+      <c r="E12">
+        <v>1000</v>
+      </c>
+      <c r="F12">
+        <v>1000</v>
+      </c>
+      <c r="G12">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13">
+        <v>1000</v>
+      </c>
+      <c r="C13">
+        <v>1000</v>
+      </c>
+      <c r="D13">
+        <v>1000</v>
+      </c>
+      <c r="E13">
+        <v>1000</v>
+      </c>
+      <c r="F13">
+        <v>1000</v>
+      </c>
+      <c r="G13">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <v>1000</v>
+      </c>
+      <c r="C14">
+        <v>1000</v>
+      </c>
+      <c r="D14">
+        <v>1000</v>
+      </c>
+      <c r="E14">
+        <v>1000</v>
+      </c>
+      <c r="F14">
+        <v>1000</v>
+      </c>
+      <c r="G14">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15">
+        <v>1000</v>
+      </c>
+      <c r="C15">
+        <v>1000</v>
+      </c>
+      <c r="D15">
+        <v>1000</v>
+      </c>
+      <c r="E15">
+        <v>1000</v>
+      </c>
+      <c r="F15">
+        <v>1000</v>
+      </c>
+      <c r="G15">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>1000</v>
+      </c>
+      <c r="C16">
+        <v>1000</v>
+      </c>
+      <c r="D16">
+        <v>1000</v>
+      </c>
+      <c r="E16">
+        <v>1000</v>
+      </c>
+      <c r="F16">
+        <v>1000</v>
+      </c>
+      <c r="G16">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17">
+        <v>1000</v>
+      </c>
+      <c r="C17">
+        <v>1000</v>
+      </c>
+      <c r="D17">
+        <v>1000</v>
+      </c>
+      <c r="E17">
+        <v>1000</v>
+      </c>
+      <c r="F17">
+        <v>1000</v>
+      </c>
+      <c r="G17">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18">
+        <v>1000</v>
+      </c>
+      <c r="C18">
+        <v>1000</v>
+      </c>
+      <c r="D18">
+        <v>1000</v>
+      </c>
+      <c r="E18">
+        <v>1000</v>
+      </c>
+      <c r="F18">
+        <v>1000</v>
+      </c>
+      <c r="G18">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19">
+        <v>1000</v>
+      </c>
+      <c r="C19">
+        <v>1000</v>
+      </c>
+      <c r="D19">
+        <v>1000</v>
+      </c>
+      <c r="E19">
+        <v>1000</v>
+      </c>
+      <c r="F19">
+        <v>1000</v>
+      </c>
+      <c r="G19">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20">
+        <v>1000</v>
+      </c>
+      <c r="C20">
+        <v>1000</v>
+      </c>
+      <c r="D20">
+        <v>1000</v>
+      </c>
+      <c r="E20">
+        <v>1000</v>
+      </c>
+      <c r="F20">
+        <v>1000</v>
+      </c>
+      <c r="G20">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21">
+        <v>1000</v>
+      </c>
+      <c r="C21">
+        <v>1000</v>
+      </c>
+      <c r="D21">
+        <v>1000</v>
+      </c>
+      <c r="E21">
+        <v>1000</v>
+      </c>
+      <c r="F21">
+        <v>1000</v>
+      </c>
+      <c r="G21">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22">
+        <v>1000</v>
+      </c>
+      <c r="C22">
+        <v>1000</v>
+      </c>
+      <c r="D22">
+        <v>1000</v>
+      </c>
+      <c r="E22">
+        <v>1000</v>
+      </c>
+      <c r="F22">
+        <v>1000</v>
+      </c>
+      <c r="G22">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23">
+        <v>1000</v>
+      </c>
+      <c r="C23">
+        <v>1000</v>
+      </c>
+      <c r="D23">
+        <v>1000</v>
+      </c>
+      <c r="E23">
+        <v>1000</v>
+      </c>
+      <c r="F23">
+        <v>1000</v>
+      </c>
+      <c r="G23">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24">
+        <v>1000</v>
+      </c>
+      <c r="C24">
+        <v>1000</v>
+      </c>
+      <c r="D24">
+        <v>1000</v>
+      </c>
+      <c r="E24">
+        <v>1000</v>
+      </c>
+      <c r="F24">
+        <v>1000</v>
+      </c>
+      <c r="G24">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25">
+        <v>1000</v>
+      </c>
+      <c r="C25">
+        <v>1000</v>
+      </c>
+      <c r="D25">
+        <v>1000</v>
+      </c>
+      <c r="E25">
+        <v>1000</v>
+      </c>
+      <c r="F25">
+        <v>1000</v>
+      </c>
+      <c r="G25">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26">
+        <v>1000</v>
+      </c>
+      <c r="C26">
+        <v>1000</v>
+      </c>
+      <c r="D26">
+        <v>1000</v>
+      </c>
+      <c r="E26">
+        <v>1000</v>
+      </c>
+      <c r="F26">
+        <v>1000</v>
+      </c>
+      <c r="G26">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27">
+        <v>1000</v>
+      </c>
+      <c r="C27">
+        <v>1000</v>
+      </c>
+      <c r="D27">
+        <v>1000</v>
+      </c>
+      <c r="E27">
+        <v>1000</v>
+      </c>
+      <c r="F27">
+        <v>1000</v>
+      </c>
+      <c r="G27">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28">
+        <v>1000</v>
+      </c>
+      <c r="C28">
+        <v>1000</v>
+      </c>
+      <c r="D28">
+        <v>1000</v>
+      </c>
+      <c r="E28">
+        <v>1000</v>
+      </c>
+      <c r="F28">
+        <v>1000</v>
+      </c>
+      <c r="G28">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29">
+        <v>1000</v>
+      </c>
+      <c r="C29">
+        <v>1000</v>
+      </c>
+      <c r="D29">
+        <v>1000</v>
+      </c>
+      <c r="E29">
+        <v>1000</v>
+      </c>
+      <c r="F29">
+        <v>1000</v>
+      </c>
+      <c r="G29">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30">
+        <v>1000</v>
+      </c>
+      <c r="C30">
+        <v>1000</v>
+      </c>
+      <c r="D30">
+        <v>1000</v>
+      </c>
+      <c r="E30">
+        <v>1000</v>
+      </c>
+      <c r="F30">
+        <v>1000</v>
+      </c>
+      <c r="G30">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31">
+        <v>1000</v>
+      </c>
+      <c r="C31">
+        <v>1000</v>
+      </c>
+      <c r="D31">
+        <v>1000</v>
+      </c>
+      <c r="E31">
+        <v>1000</v>
+      </c>
+      <c r="F31">
+        <v>1000</v>
+      </c>
+      <c r="G31">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>21</v>
+      </c>
+      <c r="B32">
+        <v>1000</v>
+      </c>
+      <c r="C32">
+        <v>1000</v>
+      </c>
+      <c r="D32">
+        <v>1000</v>
+      </c>
+      <c r="E32">
+        <v>1000</v>
+      </c>
+      <c r="F32">
+        <v>1000</v>
+      </c>
+      <c r="G32">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33">
+        <v>1000</v>
+      </c>
+      <c r="C33">
+        <v>1000</v>
+      </c>
+      <c r="D33">
+        <v>1000</v>
+      </c>
+      <c r="E33">
+        <v>1000</v>
+      </c>
+      <c r="F33">
+        <v>1000</v>
+      </c>
+      <c r="G33">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>